<commit_message>
Transitions: subtask rule, Closed Won ticket check, master Read Me notes
- team-rules.md: "Subtask - [person]" tasks are main tasks and must be
  linked to the ticket; only checklist subtasks must not be (rule 3).
  New rule 5 / record_checks: every deal that moved to Closed won
  (White Label Storage SALES) in the window has an Onboarding Pipeline
  ticket. Went-live property confirmed the same as CS Ops (live = Yes).
- Master rules Read Me: built from the live settings on 2026-10-13; the
  Go-Live Execution queue fix on 2026-10-06 was a planned change.
- Weekly audit: generic record_checks (fetch, question 1 problems with a
  link to each record, page table); documented in SKILL.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017uf8FUtnaXSoM3iiDFsscT
</commit_message>
<xml_diff>
--- a/audits/transitions-workflow-audit/Transitions_Master_Rules.xlsx
+++ b/audits/transitions-workflow-audit/Transitions_Master_Rules.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -485,6 +485,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -517,7 +518,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13 10:43 UTC (saved settings snapshot)</t>
+          <t>The live settings on 2026-10-13 (read-only snapshot taken at 10:43 UTC).</t>
         </is>
       </c>
     </row>
@@ -644,12 +645,24 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Planned change</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Go-Live Execution Tasks (+SubTask) (1866664222): on 2026-10-06 the Transitions queue (13519270) was set on its 5 Create task actions (revision 54 -&gt; 60). This was a planned change (confirmed by Cherine on 2026-10-06), so it is part of this baseline, not a change to report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Change log</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>2026-10-13: file created.</t>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13: file created from the live settings on 2026-10-13.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Transitions: Closed Won 8 Oct edit is a change not yet confirmed (W-4)
- Master rules file: the Closed Won row (1670039203) holds revision 13
  (before the 8 Oct edit), not the live settings; Read Me says so and
  the change log records why.
- team-rules.md: the edit is listed under Changes not yet confirmed and
  as Waiting on Cherine W-4, with the question, the workflow link and
  what it affects.
- describe.py: Create record actions are described in full, including
  every association and its label, so a removed association shows as a
  change instead of only a revision bump. The weekly fetch now loads
  ticket and deal association labels.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017uf8FUtnaXSoM3iiDFsscT
</commit_message>
<xml_diff>
--- a/audits/transitions-workflow-audit/Transitions_Master_Rules.xlsx
+++ b/audits/transitions-workflow-audit/Transitions_Master_Rules.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -518,7 +517,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>The live settings on 2026-10-13 (read-only snapshot taken at 10:43 UTC).</t>
+          <t>The live settings on 2026-10-13 (read-only snapshot taken at 10:43 UTC), except Closed Won (1670039203): its row holds its settings before the 8 Oct edit (revision 13), because that edit is not confirmed.</t>
         </is>
       </c>
     </row>
@@ -663,6 +662,18 @@
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>2026-10-13: file created from the live settings on 2026-10-13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13: updated 1670039203. Closed Won (1670039203) row set to its settings before the 8 Oct edit (revision 13, read 2026-10-06). The 8 Oct edit (revision 14: no longer copies the deal's companies onto the ticket) is not confirmed (Cherine, 2026-10-13), so it is reported as a change, not yet confirmed (Waiting on Cherine W-4).</t>
         </is>
       </c>
     </row>
@@ -821,7 +832,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>When a deal reaches Closed won (White Label Storage SALES pipeline), creates one Onboarding Pipeline ticket in UNASSIGNED named after the deal, owned by Elizabeth Airey, linked to the deal and the deal's contacts. Creates no tasks.</t>
+          <t>When a deal reaches Closed won (White Label Storage SALES pipeline), creates one Onboarding Pipeline ticket in UNASSIGNED named after the deal, owned by Elizabeth Airey, linked to the deal, the deal's contacts and the deal's companies (label "Transitions"). Creates no tasks. Baseline = revision 13; the 8 Oct edit (revision 14) is not confirmed.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -856,7 +867,7 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>(start): Create record - {"associations": [{"target": {"associationCategory": "HUBSPOT_DEFINED", "associationTypeId": 16}, "value": {"sourceSpec": {"associationCategory": "HUBSPOT_DEFINED", "associationTypeId": 3}, "type": "C</t>
+          <t>(start): Create record - create a Ticket; set Ticket name = {{ enrolled_object.dealname }}; Ticket status = UNASSIGNED; Ticket owner = Elizabeth Airey; links: Ticket -&gt; Contact (all): copied from the enrolled record's Deal -&gt; Contact (all); Ticket -&gt; Company, label "Transitions": copied from the enrolled record's Deal -&gt; Company (all); Ticket -&gt; Deal (all): the enrolled record</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
@@ -881,12 +892,12 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08 11:35:19 UTC</t>
+          <t>2026-07-15 11:06:08 UTC</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr"/>
@@ -1615,7 +1626,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","actionTypeId":"0-14","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":16},"value":{"sourceSpec":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":3},"type":"COPY_ASSOCIATION"}},{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":28},"value":{"type":"ENROLLED_OBJECT"}}],"object_type_id":"0-5","properties":[{"targetProperty":"subject","value":{"staticValue":"{{ enrolled_object.dealname }}","type":"STATIC_VALUE"}},{"targetProperty":"hs_pipeline_stage","value":{"staticValue":"1100007030","type":"STATIC_VALUE"}},{"targetProperty":"hubspot_owner_id","value":{"staticValue":"81929768","type":"STATIC_VALUE"}}],"use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["150102819"]},"property":"dealstage"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":false,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"id":"1670039203","isEnabled":true,"name":"Closed Won | Create Ticket in INITIAL SETUP - UNASSIGNED","objectTypeId":"0-3","revisionId":"14","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T11:35:19.692Z"}</t>
+          <t>{"actions":[{"actionId":"1","actionTypeId":"0-14","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":16},"value":{"sourceSpec":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":3},"type":"COPY_ASSOCIATION"}},{"target":{"associationCategory":"USER_DEFINED","associationTypeId":70},"value":{"sourceSpec":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":341},"type":"COPY_ASSOCIATION"}},{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":28},"value":{"type":"ENROLLED_OBJECT"}}],"object_type_id":"0-5","properties":[{"targetProperty":"subject","value":{"staticValue":"{{ enrolled_object.dealname }}","type":"STATIC_VALUE"}},{"targetProperty":"hs_pipeline_stage","value":{"staticValue":"1100007030","type":"STATIC_VALUE"}},{"targetProperty":"hubspot_owner_id","value":{"staticValue":"81929768","type":"STATIC_VALUE"}}],"use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["150102819"]},"property":"dealstage"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":false,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"id":"1670039203","isEnabled":true,"name":"Closed Won | Create Ticket in INITIAL SETUP - UNASSIGNED","objectTypeId":"0-3","revisionId":"13","startActionId":"1","timeWindows":[],"updatedAt":"2026-07-15T11:06:08.153Z"}</t>
         </is>
       </c>
     </row>

</xml_diff>